<commit_message>
Save all pending audit workflows, evidence, and workbook changes
</commit_message>
<xml_diff>
--- a/Tools/Накази.xlsx
+++ b/Tools/Накази.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ЦяКнига" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Справки\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Строевые приказы\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DE90A7-B305-4F0A-AE10-698FB5AE8EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C683896-110A-4542-9234-345F288BAA9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FF16710E-FAF6-445F-AD75-CD3560A0E894}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="452" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="12">
   <si>
     <t>Дата наказу</t>
   </si>
@@ -236,7 +236,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 4" xfId="1" xr:uid="{98265266-0594-4C2A-BAC9-F7BD39857057}"/>
   </cellStyles>
   <dxfs count="25">
@@ -770,9 +770,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -810,7 +810,7 @@
         <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
@@ -916,7 +916,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -6223,7 +6223,9 @@
       <c r="F278" s="2">
         <v>276</v>
       </c>
-      <c r="G278" s="9"/>
+      <c r="G278" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A279" s="3">
@@ -6241,7 +6243,9 @@
       <c r="F279" s="2">
         <v>277</v>
       </c>
-      <c r="G279" s="9"/>
+      <c r="G279" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A280" s="3">
@@ -6259,7 +6263,9 @@
       <c r="F280" s="2">
         <v>278</v>
       </c>
-      <c r="G280" s="9"/>
+      <c r="G280" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A281" s="3">
@@ -6277,7 +6283,9 @@
       <c r="F281" s="2">
         <v>279</v>
       </c>
-      <c r="G281" s="9"/>
+      <c r="G281" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A282" s="3">
@@ -6295,7 +6303,9 @@
       <c r="F282" s="2">
         <v>280</v>
       </c>
-      <c r="G282" s="9"/>
+      <c r="G282" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A283" s="3">
@@ -6313,7 +6323,9 @@
       <c r="F283" s="2">
         <v>281</v>
       </c>
-      <c r="G283" s="9"/>
+      <c r="G283" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A284" s="3">
@@ -6331,7 +6343,9 @@
       <c r="F284" s="2">
         <v>282</v>
       </c>
-      <c r="G284" s="9"/>
+      <c r="G284" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A285" s="3">
@@ -6349,7 +6363,9 @@
       <c r="F285" s="2">
         <v>283</v>
       </c>
-      <c r="G285" s="9"/>
+      <c r="G285" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="286" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A286" s="3">
@@ -6367,7 +6383,9 @@
       <c r="F286" s="2">
         <v>284</v>
       </c>
-      <c r="G286" s="9"/>
+      <c r="G286" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A287" s="3">
@@ -6385,7 +6403,9 @@
       <c r="F287" s="2">
         <v>285</v>
       </c>
-      <c r="G287" s="9"/>
+      <c r="G287" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A288" s="3">
@@ -6403,7 +6423,9 @@
       <c r="F288" s="2">
         <v>286</v>
       </c>
-      <c r="G288" s="9"/>
+      <c r="G288" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A289" s="3">
@@ -6421,7 +6443,9 @@
       <c r="F289" s="2">
         <v>287</v>
       </c>
-      <c r="G289" s="9"/>
+      <c r="G289" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A290" s="3">
@@ -6439,7 +6463,9 @@
       <c r="F290" s="2">
         <v>288</v>
       </c>
-      <c r="G290" s="9"/>
+      <c r="G290" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A291" s="3">
@@ -6457,7 +6483,9 @@
       <c r="F291" s="2">
         <v>289</v>
       </c>
-      <c r="G291" s="9"/>
+      <c r="G291" s="6" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A292" s="3">

</xml_diff>

<commit_message>
Update food report workflow, templates and extract generation
</commit_message>
<xml_diff>
--- a/Tools/Накази.xlsx
+++ b/Tools/Накази.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WORK\Windows\Строевые приказы\Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46A8383-69C3-4514-8EA1-4E6CCA3AF1B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A45768-D5DB-492C-A571-1EBA7176F122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FF16710E-FAF6-445F-AD75-CD3560A0E894}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1817" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1892" uniqueCount="21">
   <si>
     <t>Дата наказу</t>
   </si>
@@ -293,367 +293,36 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Обычный 4" xfId="1" xr:uid="{98265266-0594-4C2A-BAC9-F7BD39857057}"/>
   </cellStyles>
-  <dxfs count="46">
+  <dxfs count="36">
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -813,147 +482,10 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color indexed="64"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -967,6 +499,16 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -1006,6 +548,364 @@
         </right>
         <top/>
         <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
       </border>
     </dxf>
     <dxf>
@@ -1114,14 +1014,14 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="TableStyleDark_my" pivot="0" count="8" xr9:uid="{CFC3E1FC-0CEF-4FBB-AEF8-B86D335BF785}">
-      <tableStyleElement type="wholeTable" dxfId="45"/>
-      <tableStyleElement type="headerRow" dxfId="44"/>
-      <tableStyleElement type="totalRow" dxfId="43"/>
-      <tableStyleElement type="firstColumn" dxfId="42"/>
-      <tableStyleElement type="lastColumn" dxfId="41"/>
-      <tableStyleElement type="firstRowStripe" dxfId="40"/>
-      <tableStyleElement type="secondRowStripe" dxfId="39"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="38"/>
+      <tableStyleElement type="wholeTable" dxfId="35"/>
+      <tableStyleElement type="headerRow" dxfId="34"/>
+      <tableStyleElement type="totalRow" dxfId="33"/>
+      <tableStyleElement type="firstColumn" dxfId="32"/>
+      <tableStyleElement type="lastColumn" dxfId="31"/>
+      <tableStyleElement type="firstRowStripe" dxfId="30"/>
+      <tableStyleElement type="secondRowStripe" dxfId="29"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="28"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1136,38 +1036,38 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E5B67A-5EFE-4A5D-B6E9-77A9B6EC75CB}" name="tbMapNumberOrderToDate2025" displayName="tbMapNumberOrderToDate2025" ref="A2:C384" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F7E5B67A-5EFE-4A5D-B6E9-77A9B6EC75CB}" name="tbMapNumberOrderToDate2025" displayName="tbMapNumberOrderToDate2025" ref="A2:C384" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
   <autoFilter ref="A2:C384" xr:uid="{F7E5B67A-5EFE-4A5D-B6E9-77A9B6EC75CB}"/>
   <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{B697DAFA-710E-4CD5-A7FB-D72CC37C846A}" name="Дата наказу" dataDxfId="2"/>
-    <tableColumn id="1" xr3:uid="{32AB775B-7E00-4ABD-B4CC-80D52F6BA667}" name="Номер наказу" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{BC4631F7-FFE6-4688-B2C0-D9F319889EA5}" name="Підписант" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{B697DAFA-710E-4CD5-A7FB-D72CC37C846A}" name="Дата наказу" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{32AB775B-7E00-4ABD-B4CC-80D52F6BA667}" name="Номер наказу" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{BC4631F7-FFE6-4688-B2C0-D9F319889EA5}" name="Підписант" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark_my" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{209B9E54-E3CC-4D8D-BA91-F407DFC7AF17}" name="tbMapNumberOrderToDate" displayName="tbMapNumberOrderToDate" ref="E2:G384" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13" totalsRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{209B9E54-E3CC-4D8D-BA91-F407DFC7AF17}" name="tbMapNumberOrderToDate" displayName="tbMapNumberOrderToDate" ref="E2:G384" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="18" tableBorderDxfId="17" totalsRowBorderDxfId="16">
   <autoFilter ref="E2:G384" xr:uid="{209B9E54-E3CC-4D8D-BA91-F407DFC7AF17}"/>
   <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{33899C36-507D-430B-9FEA-342619068B10}" name="Дата наказу" dataDxfId="10"/>
-    <tableColumn id="1" xr3:uid="{00D54055-9EDB-4EE5-93B4-E80DEBA7BA0C}" name="Номер наказу" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{F2E7A201-8655-4C78-B1C4-9C74E6A9A8B9}" name="Підписант" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{33899C36-507D-430B-9FEA-342619068B10}" name="Дата наказу" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{00D54055-9EDB-4EE5-93B4-E80DEBA7BA0C}" name="Номер наказу" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{F2E7A201-8655-4C78-B1C4-9C74E6A9A8B9}" name="Підписант" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark_my" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EDF8C4E6-3A95-4DD9-85F9-157DC8B1CCDD}" name="tbOrders" displayName="tbOrders" ref="J2:N555" totalsRowShown="0" headerRowDxfId="37" dataDxfId="15" headerRowBorderDxfId="35" tableBorderDxfId="36" totalsRowBorderDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EDF8C4E6-3A95-4DD9-85F9-157DC8B1CCDD}" name="tbOrders" displayName="tbOrders" ref="J2:N555" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <autoFilter ref="J2:N555" xr:uid="{EDF8C4E6-3A95-4DD9-85F9-157DC8B1CCDD}"/>
   <tableColumns count="5">
-    <tableColumn id="4" xr3:uid="{DA43EE14-2E47-42B6-BD3B-9B8A7CFA6EE4}" name="Дата" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{E8A30FAA-0CC3-4C9E-BA3C-8BE0DDE07B86}" name="Номер наказа" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{1ED0B052-C95F-4A20-BD03-DFE4CA46CE3D}" name="Підписант" dataDxfId="18"/>
-    <tableColumn id="1" xr3:uid="{7584F36D-3DA5-4400-B180-3B7D4F52FA5E}" name="ПІБ" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{F93BF2F9-E4D9-4ECB-9930-1DF3B93C689F}" name="Звання" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{DA43EE14-2E47-42B6-BD3B-9B8A7CFA6EE4}" name="Дата" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{E8A30FAA-0CC3-4C9E-BA3C-8BE0DDE07B86}" name="Номер наказа" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{1ED0B052-C95F-4A20-BD03-DFE4CA46CE3D}" name="Підписант" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{7584F36D-3DA5-4400-B180-3B7D4F52FA5E}" name="ПІБ" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{F93BF2F9-E4D9-4ECB-9930-1DF3B93C689F}" name="Звання" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark_my" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -15254,9 +15154,15 @@
       <c r="K463" s="13">
         <v>290</v>
       </c>
-      <c r="L463" s="12"/>
-      <c r="M463" s="17"/>
-      <c r="N463" s="17"/>
+      <c r="L463" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M463" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N463" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="464" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J464" s="12">
@@ -15265,9 +15171,15 @@
       <c r="K464" s="13">
         <v>291</v>
       </c>
-      <c r="L464" s="12"/>
-      <c r="M464" s="17"/>
-      <c r="N464" s="17"/>
+      <c r="L464" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M464" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N464" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="465" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J465" s="12">
@@ -15276,9 +15188,15 @@
       <c r="K465" s="13">
         <v>292</v>
       </c>
-      <c r="L465" s="12"/>
-      <c r="M465" s="17"/>
-      <c r="N465" s="17"/>
+      <c r="L465" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M465" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N465" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="466" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J466" s="12">
@@ -15287,9 +15205,15 @@
       <c r="K466" s="13">
         <v>293</v>
       </c>
-      <c r="L466" s="12"/>
-      <c r="M466" s="17"/>
-      <c r="N466" s="17"/>
+      <c r="L466" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M466" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N466" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="467" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J467" s="12">
@@ -15298,9 +15222,15 @@
       <c r="K467" s="13">
         <v>294</v>
       </c>
-      <c r="L467" s="12"/>
-      <c r="M467" s="17"/>
-      <c r="N467" s="17"/>
+      <c r="L467" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M467" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N467" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="468" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J468" s="12">
@@ -15309,9 +15239,15 @@
       <c r="K468" s="13">
         <v>295</v>
       </c>
-      <c r="L468" s="12"/>
-      <c r="M468" s="17"/>
-      <c r="N468" s="17"/>
+      <c r="L468" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M468" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N468" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="469" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J469" s="12">
@@ -15320,9 +15256,15 @@
       <c r="K469" s="13">
         <v>296</v>
       </c>
-      <c r="L469" s="12"/>
-      <c r="M469" s="17"/>
-      <c r="N469" s="17"/>
+      <c r="L469" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M469" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N469" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="470" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J470" s="12">
@@ -15331,9 +15273,15 @@
       <c r="K470" s="13">
         <v>297</v>
       </c>
-      <c r="L470" s="12"/>
-      <c r="M470" s="17"/>
-      <c r="N470" s="17"/>
+      <c r="L470" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M470" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N470" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="471" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J471" s="12">
@@ -15342,9 +15290,15 @@
       <c r="K471" s="13">
         <v>298</v>
       </c>
-      <c r="L471" s="12"/>
-      <c r="M471" s="17"/>
-      <c r="N471" s="17"/>
+      <c r="L471" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M471" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N471" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="472" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J472" s="12">
@@ -15353,9 +15307,15 @@
       <c r="K472" s="13">
         <v>299</v>
       </c>
-      <c r="L472" s="12"/>
-      <c r="M472" s="17"/>
-      <c r="N472" s="17"/>
+      <c r="L472" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M472" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N472" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="473" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J473" s="12">
@@ -15364,107 +15324,253 @@
       <c r="K473" s="13">
         <v>300</v>
       </c>
-      <c r="L473" s="12"/>
-      <c r="M473" s="17"/>
-      <c r="N473" s="17"/>
+      <c r="L473" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M473" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N473" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="474" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J474" s="12"/>
-      <c r="K474" s="13"/>
-      <c r="L474" s="12"/>
-      <c r="M474" s="17"/>
-      <c r="N474" s="17"/>
+      <c r="J474" s="12">
+        <v>46313</v>
+      </c>
+      <c r="K474" s="13">
+        <v>301</v>
+      </c>
+      <c r="L474" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M474" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N474" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="475" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J475" s="12"/>
-      <c r="K475" s="13"/>
-      <c r="L475" s="12"/>
-      <c r="M475" s="17"/>
-      <c r="N475" s="17"/>
+      <c r="J475" s="12">
+        <v>46314</v>
+      </c>
+      <c r="K475" s="13">
+        <v>302</v>
+      </c>
+      <c r="L475" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M475" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N475" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="476" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J476" s="12"/>
-      <c r="K476" s="13"/>
-      <c r="L476" s="12"/>
-      <c r="M476" s="17"/>
-      <c r="N476" s="17"/>
+      <c r="J476" s="12">
+        <v>46315</v>
+      </c>
+      <c r="K476" s="13">
+        <v>303</v>
+      </c>
+      <c r="L476" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M476" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N476" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="477" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J477" s="12"/>
-      <c r="K477" s="13"/>
-      <c r="L477" s="12"/>
-      <c r="M477" s="17"/>
-      <c r="N477" s="17"/>
+      <c r="J477" s="12">
+        <v>46316</v>
+      </c>
+      <c r="K477" s="13">
+        <v>304</v>
+      </c>
+      <c r="L477" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M477" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N477" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="478" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J478" s="12"/>
-      <c r="K478" s="13"/>
-      <c r="L478" s="12"/>
-      <c r="M478" s="17"/>
-      <c r="N478" s="17"/>
+      <c r="J478" s="12">
+        <v>46317</v>
+      </c>
+      <c r="K478" s="13">
+        <v>305</v>
+      </c>
+      <c r="L478" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M478" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N478" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="479" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J479" s="12"/>
-      <c r="K479" s="13"/>
-      <c r="L479" s="12"/>
-      <c r="M479" s="17"/>
-      <c r="N479" s="17"/>
+      <c r="J479" s="12">
+        <v>46318</v>
+      </c>
+      <c r="K479" s="13">
+        <v>306</v>
+      </c>
+      <c r="L479" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M479" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N479" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="480" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J480" s="12"/>
-      <c r="K480" s="13"/>
-      <c r="L480" s="12"/>
-      <c r="M480" s="17"/>
-      <c r="N480" s="17"/>
+      <c r="J480" s="12">
+        <v>46319</v>
+      </c>
+      <c r="K480" s="13">
+        <v>307</v>
+      </c>
+      <c r="L480" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M480" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N480" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="481" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J481" s="12"/>
-      <c r="K481" s="13"/>
-      <c r="L481" s="12"/>
-      <c r="M481" s="17"/>
-      <c r="N481" s="17"/>
+      <c r="J481" s="12">
+        <v>46320</v>
+      </c>
+      <c r="K481" s="13">
+        <v>308</v>
+      </c>
+      <c r="L481" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M481" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N481" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="482" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J482" s="12"/>
-      <c r="K482" s="13"/>
-      <c r="L482" s="12"/>
-      <c r="M482" s="17"/>
-      <c r="N482" s="17"/>
+      <c r="J482" s="12">
+        <v>46321</v>
+      </c>
+      <c r="K482" s="13">
+        <v>309</v>
+      </c>
+      <c r="L482" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M482" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N482" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="483" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J483" s="12"/>
-      <c r="K483" s="13"/>
-      <c r="L483" s="12"/>
-      <c r="M483" s="17"/>
-      <c r="N483" s="17"/>
+      <c r="J483" s="12">
+        <v>46322</v>
+      </c>
+      <c r="K483" s="13">
+        <v>310</v>
+      </c>
+      <c r="L483" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M483" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N483" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="484" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J484" s="12"/>
-      <c r="K484" s="13"/>
-      <c r="L484" s="12"/>
-      <c r="M484" s="17"/>
-      <c r="N484" s="17"/>
+      <c r="J484" s="12">
+        <v>46323</v>
+      </c>
+      <c r="K484" s="13">
+        <v>311</v>
+      </c>
+      <c r="L484" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M484" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N484" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="485" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J485" s="12"/>
-      <c r="K485" s="13"/>
-      <c r="L485" s="12"/>
-      <c r="M485" s="17"/>
-      <c r="N485" s="17"/>
+      <c r="J485" s="12">
+        <v>46324</v>
+      </c>
+      <c r="K485" s="13">
+        <v>312</v>
+      </c>
+      <c r="L485" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M485" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N485" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="486" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J486" s="12"/>
-      <c r="K486" s="13"/>
-      <c r="L486" s="12"/>
-      <c r="M486" s="17"/>
-      <c r="N486" s="17"/>
+      <c r="J486" s="12">
+        <v>46325</v>
+      </c>
+      <c r="K486" s="13">
+        <v>313</v>
+      </c>
+      <c r="L486" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M486" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N486" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="487" spans="10:14" x14ac:dyDescent="0.25">
-      <c r="J487" s="12"/>
-      <c r="K487" s="13"/>
-      <c r="L487" s="12"/>
-      <c r="M487" s="17"/>
-      <c r="N487" s="17"/>
+      <c r="J487" s="12">
+        <v>46326</v>
+      </c>
+      <c r="K487" s="13">
+        <v>314</v>
+      </c>
+      <c r="L487" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="M487" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="N487" s="16" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="488" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J488" s="12"/>
@@ -15945,13 +16051,13 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="A3:A384">
-    <cfRule type="duplicateValues" dxfId="26" priority="1015"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1015"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E384">
-    <cfRule type="duplicateValues" dxfId="25" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J555">
-    <cfRule type="duplicateValues" dxfId="24" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="3">

</xml_diff>